<commit_message>
Ajout du style pour toutes les pages + redirection des bouttons
</commit_message>
<xml_diff>
--- a/assets/pdf/tableau des copmpétences.xlsx
+++ b/assets/pdf/tableau des copmpétences.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninoh\Desktop\nino.github.io\assets\pdf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAC68FCA-1065-4A6F-82F3-512F63E078DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B647AB5-8218-47CE-A545-B35F8EFB4D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -98,9 +98,6 @@
 (intitulé et liste des documents et productions associés)</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
   </si>
   <si>
@@ -110,12 +107,6 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :</t>
-  </si>
-  <si>
-    <t>SESSION 2023</t>
-  </si>
-  <si>
     <t>X SISR</t>
   </si>
   <si>
@@ -128,12 +119,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>Projet de HACKATON</t>
-  </si>
-  <si>
-    <t>Du 6/11/2025 au 6/11/2025</t>
-  </si>
-  <si>
     <t>Mise à jour constante du parc informatique (GLPI)</t>
   </si>
   <si>
@@ -155,12 +140,6 @@
     <t>Installation et configuration de borne d'acceuil pour acceuil public</t>
   </si>
   <si>
-    <t>Travaux pratiques Active Directory</t>
-  </si>
-  <si>
-    <t>Projet de BLACK BASTION</t>
-  </si>
-  <si>
     <t>02/09/2024 au 31/08/2025</t>
   </si>
   <si>
@@ -170,16 +149,64 @@
     <t>Préparation de plusieurs postes d'inspecteurs</t>
   </si>
   <si>
-    <t>Travaux pratiques noté GLPI</t>
-  </si>
-  <si>
-    <t>Du 2/11/2025 à Indéfinie</t>
-  </si>
-  <si>
-    <t>Du 9/10/2025 au 16/10/2025</t>
-  </si>
-  <si>
-    <t>Du 13/11/2025 au 25/01/2026</t>
+    <t>02/09/2024 - 15/05/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestion et administration d'une forêt Active Directory </t>
+  </si>
+  <si>
+    <t>Déploiement d'une solution de gestion des tickets GLPI</t>
+  </si>
+  <si>
+    <t>Gérer une équipe en mode projet (hackathon)</t>
+  </si>
+  <si>
+    <t>Déployer un site internet pour la présence en ligne du projet hackathon</t>
+  </si>
+  <si>
+    <t>Mise en place d'une infrastructure réseau</t>
+  </si>
+  <si>
+    <t>Schématiser une infrastructure informatique</t>
+  </si>
+  <si>
+    <t>Création de mon portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Securisation d'une infrastructure avec un IDS/IPS avec Suricata </t>
+  </si>
+  <si>
+    <t>Référencer les besoins d'un système d'information pour le projet hackathon</t>
+  </si>
+  <si>
+    <t>Automatisation de déploiement de pare-feu pfsense</t>
+  </si>
+  <si>
+    <t>Réintégration d'utilisateur et poste dans l'Active Directory</t>
+  </si>
+  <si>
+    <t>Gestions de droit d'accès utilisateur</t>
+  </si>
+  <si>
+    <t>Formation des stagiaires</t>
+  </si>
+  <si>
+    <t>Formation des nouveaux alternants</t>
+  </si>
+  <si>
+    <t>Projet migration version office pour inspecteur (32 vers 64 bit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet d'arrivée massive </t>
+  </si>
+  <si>
+    <t>N° candidat : 2249710472</t>
+  </si>
+  <si>
+    <t>SESSION 2026</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://trabdor1.github.io/nino.github.io/index.html</t>
   </si>
 </sst>
 </file>
@@ -252,12 +279,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="30">
@@ -666,7 +705,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -704,9 +743,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -734,9 +770,48 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -761,44 +836,21 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1111,7 +1163,7 @@
   <dimension ref="A1:AQ81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.90625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.453125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="95.453125" style="1" customWidth="1"/>
     <col min="2" max="2" width="35.90625" style="1" customWidth="1"/>
     <col min="3" max="8" width="18.6328125" style="1" customWidth="1"/>
     <col min="9" max="43" width="11.453125" customWidth="1"/>
@@ -1119,84 +1171,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="31"/>
+      <c r="A3" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="14" t="s">
+      <c r="A4" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="21" t="s">
+      <c r="G4" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
+      <c r="A5" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="40" t="s">
-        <v>19</v>
+      <c r="B6" s="31" t="s">
+        <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1218,8 +1270,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33"/>
-      <c r="B7" s="41"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1275,16 +1327,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="27"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1321,23 +1373,19 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="17"/>
-      <c r="H9" s="18"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="45"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="17"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1374,21 +1422,19 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="18"/>
+      <c r="B10" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="45"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="17"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1425,21 +1471,19 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="47"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1476,21 +1520,19 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="17"/>
-      <c r="H12" s="18"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1527,15 +1569,19 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="18"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="46"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="17"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1572,15 +1618,19 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="18"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="46"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="17"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1617,15 +1667,19 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="47"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1662,15 +1716,19 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="18"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="16"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1707,15 +1765,19 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="18"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="46"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="17"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1752,15 +1814,19 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="18"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="17"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1798,16 +1864,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
+      <c r="A19" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1846,19 +1912,17 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="18"/>
+        <v>32</v>
+      </c>
+      <c r="C20" s="45"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1897,19 +1961,17 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E21" s="17"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="18"/>
+        <v>32</v>
+      </c>
+      <c r="C21" s="15"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="17"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1948,23 +2010,17 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E22" s="17"/>
-      <c r="F22" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="G22" s="17"/>
-      <c r="H22" s="18"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -2003,19 +2059,17 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
+        <v>32</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -2053,14 +2107,18 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="18"/>
+      <c r="A24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="17"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2098,14 +2156,18 @@
       <c r="AQ24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
+      <c r="A25" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2143,14 +2205,16 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11"/>
+      <c r="A26" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="B26" s="10"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="18"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2188,16 +2252,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
+      <c r="A27" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2236,21 +2300,17 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="G28" s="17"/>
-      <c r="H28" s="18"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2289,19 +2349,17 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E29" s="17"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="18"/>
+        <v>33</v>
+      </c>
+      <c r="C29" s="15"/>
+      <c r="D29" s="45"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2340,21 +2398,17 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E30" s="17"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="18"/>
+        <v>33</v>
+      </c>
+      <c r="C30" s="45"/>
+      <c r="D30" s="45"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2393,21 +2447,19 @@
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
+        <v>34</v>
+      </c>
+      <c r="B31" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="45"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2445,14 +2497,18 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="18"/>
+      <c r="A32" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="47"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2490,14 +2546,18 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="18"/>
+      <c r="A33" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="47"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2535,14 +2595,18 @@
       <c r="AQ33"/>
     </row>
     <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="12"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="20"/>
+      <c r="A34" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="19"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2672,6 +2736,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2679,11 +2748,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2694,23 +2758,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="923fc38d-de99-4f41-a854-2ef3d7139c32" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FA205DCF765DAB4DA1320CF954065217" ma:contentTypeVersion="6" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="09f44f9abc05b590af14fb2003245ed6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="923fc38d-de99-4f41-a854-2ef3d7139c32" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="832122d8c8a8cfd2593c13827068e246" ns3:_="">
     <xsd:import namespace="923fc38d-de99-4f41-a854-2ef3d7139c32"/>
@@ -2866,31 +2913,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54EE2C10-20C2-480F-89DB-8853DDCBD6C6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="923fc38d-de99-4f41-a854-2ef3d7139c32"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83E7EC4C-DC51-4E4E-8784-7DCDB7CD0416}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="923fc38d-de99-4f41-a854-2ef3d7139c32" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ABF21E1-9BD9-427B-921D-D5D8FA174013}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2906,4 +2946,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83E7EC4C-DC51-4E4E-8784-7DCDB7CD0416}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54EE2C10-20C2-480F-89DB-8853DDCBD6C6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="923fc38d-de99-4f41-a854-2ef3d7139c32"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajout des procédure pour les projets
</commit_message>
<xml_diff>
--- a/assets/pdf/tableau des copmpétences.xlsx
+++ b/assets/pdf/tableau des copmpétences.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninoh\Desktop\nino.github.io\assets\pdf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B647AB5-8218-47CE-A545-B35F8EFB4D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D09242-0FB8-47AD-A1A2-842A673DF48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="54">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>Centre de formation : EFREI Villejuif</t>
-  </si>
-  <si>
-    <t>X</t>
   </si>
   <si>
     <t>Mise à jour constante du parc informatique (GLPI)</t>
@@ -770,72 +767,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -851,6 +782,72 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1171,56 +1168,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="24"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="42" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="43"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="43"/>
+      <c r="H3" s="49"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="13" t="s">
         <v>8</v>
       </c>
@@ -1232,22 +1229,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35"/>
+      <c r="A5" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="37" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1270,8 +1267,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23"/>
-      <c r="B7" s="32"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1327,16 +1324,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1374,17 +1371,17 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="44" t="s">
-        <v>36</v>
-      </c>
-      <c r="B9" s="44" t="s">
+      <c r="A9" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="45"/>
+      <c r="B9" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="23"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="15"/>
-      <c r="G9" s="46"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="17"/>
       <c r="I9"/>
       <c r="J9"/>
@@ -1423,14 +1420,14 @@
       <c r="AQ9"/>
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="45"/>
-      <c r="D10" s="46"/>
+      <c r="A10" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="15"/>
@@ -1472,18 +1469,18 @@
       <c r="AQ10"/>
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="44" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="44" t="s">
-        <v>35</v>
+      <c r="A11" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
-      <c r="F11" s="46"/>
+      <c r="F11" s="24"/>
       <c r="G11" s="16"/>
-      <c r="H11" s="47"/>
+      <c r="H11" s="25"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1521,16 +1518,16 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="44" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="44" t="s">
-        <v>35</v>
+      <c r="A12" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="45"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="23"/>
       <c r="G12" s="16"/>
       <c r="H12" s="17"/>
       <c r="I12"/>
@@ -1570,17 +1567,17 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="44" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="46"/>
+      <c r="A13" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="24"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="17"/>
       <c r="I13"/>
       <c r="J13"/>
@@ -1619,17 +1616,17 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="46"/>
+      <c r="A14" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="24"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="48"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
       <c r="H14" s="17"/>
       <c r="I14"/>
       <c r="J14"/>
@@ -1668,18 +1665,18 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="44" t="s">
-        <v>35</v>
+      <c r="A15" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
-      <c r="H15" s="47"/>
+      <c r="H15" s="25"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1717,14 +1714,14 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="44" t="s">
-        <v>35</v>
+      <c r="A16" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="C16" s="16"/>
-      <c r="D16" s="46"/>
+      <c r="D16" s="24"/>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
@@ -1766,17 +1763,17 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="46"/>
+      <c r="A17" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="24"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
       <c r="H17" s="17"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1815,17 +1812,17 @@
       <c r="AQ17"/>
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" s="44" t="s">
-        <v>35</v>
+      <c r="A18" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>34</v>
       </c>
       <c r="C18"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
       <c r="H18" s="17"/>
       <c r="I18"/>
       <c r="J18"/>
@@ -1864,16 +1861,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="30"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1912,12 +1909,12 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="45"/>
+        <v>31</v>
+      </c>
+      <c r="C20" s="23"/>
       <c r="D20" s="15"/>
       <c r="E20" s="16"/>
       <c r="F20" s="15"/>
@@ -1961,16 +1958,16 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C21" s="15"/>
-      <c r="D21" s="45"/>
+      <c r="D21" s="23"/>
       <c r="E21" s="16"/>
       <c r="F21" s="15"/>
-      <c r="G21" s="46"/>
+      <c r="G21" s="24"/>
       <c r="H21" s="17"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -2010,13 +2007,13 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
+        <v>31</v>
+      </c>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
       <c r="E22" s="16"/>
       <c r="F22" s="15"/>
       <c r="G22" s="16"/>
@@ -2059,13 +2056,13 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="16"/>
-      <c r="D23" s="45"/>
+      <c r="D23" s="23"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
@@ -2108,16 +2105,16 @@
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" s="16"/>
-      <c r="D24" s="46"/>
+      <c r="D24" s="24"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
-      <c r="G24" s="46"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="17"/>
       <c r="I24"/>
       <c r="J24"/>
@@ -2157,13 +2154,13 @@
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25" s="16"/>
-      <c r="D25" s="46"/>
+      <c r="D25" s="24"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="16"/>
@@ -2206,13 +2203,13 @@
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
-      <c r="F26" s="46"/>
+      <c r="F26" s="24"/>
       <c r="G26" s="16"/>
       <c r="H26" s="17"/>
       <c r="I26"/>
@@ -2252,16 +2249,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="30"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2300,15 +2297,15 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" s="45"/>
+        <v>32</v>
+      </c>
+      <c r="C28" s="23"/>
       <c r="D28" s="15"/>
       <c r="E28" s="16"/>
-      <c r="F28" s="45"/>
+      <c r="F28" s="23"/>
       <c r="G28" s="16"/>
       <c r="H28" s="17"/>
       <c r="I28"/>
@@ -2349,13 +2346,13 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C29" s="15"/>
-      <c r="D29" s="45"/>
+      <c r="D29" s="23"/>
       <c r="E29" s="16"/>
       <c r="F29" s="15"/>
       <c r="G29" s="16"/>
@@ -2398,13 +2395,13 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
+        <v>32</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
       <c r="E30" s="16"/>
       <c r="F30" s="15"/>
       <c r="G30" s="16"/>
@@ -2447,17 +2444,15 @@
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="C31" s="45"/>
+        <v>32</v>
+      </c>
+      <c r="C31" s="23"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
-      <c r="F31" s="16" t="s">
-        <v>24</v>
-      </c>
+      <c r="F31" s="24"/>
       <c r="G31" s="16"/>
       <c r="H31" s="17"/>
       <c r="I31"/>
@@ -2498,17 +2493,17 @@
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
       <c r="F32" s="16"/>
       <c r="G32" s="16"/>
-      <c r="H32" s="47"/>
+      <c r="H32" s="25"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2547,17 +2542,17 @@
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
-      <c r="H33" s="47"/>
+      <c r="H33" s="25"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2596,15 +2591,15 @@
     </row>
     <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C34" s="18"/>
       <c r="D34" s="18"/>
       <c r="E34" s="18"/>
-      <c r="F34" s="49"/>
+      <c r="F34" s="27"/>
       <c r="G34" s="18"/>
       <c r="H34" s="19"/>
       <c r="I34"/>
@@ -2752,7 +2747,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="8" scale="60" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
@@ -2959,15 +2954,15 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54EE2C10-20C2-480F-89DB-8853DDCBD6C6}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="923fc38d-de99-4f41-a854-2ef3d7139c32"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>